<commit_message>
fixed plot generation problems and simulated version fold training problem, which had the same problems for every fold in train
</commit_message>
<xml_diff>
--- a/n_puzzle_trajectory_gt_confusion.xlsx
+++ b/n_puzzle_trajectory_gt_confusion.xlsx
@@ -629,359 +629,389 @@
       <c r="C6" s="5" t="inlineStr">
         <is>
           <t>TP=5 FP=0
+FN=0 TN=0
+SW=0</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>TP=57 FP=0
+FN=1 TN=0
+SW=0</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>TP=48 FP=0
+FN=1 TN=0
+SW=0</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>TP=48 FP=0
+FN=3 TN=0
+SW=0</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>TP=162 FP=0
+FN=0 TN=0
+SW=0</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>TP=258 FP=0
+FN=0 TN=0
+SW=0</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>TP=211 FP=0
+FN=1 TN=0
+SW=0</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>TP=40 FP=0
+FN=1 TN=0
+SW=0</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>TP=297 FP=0
+FN=3 TN=0
+SW=0</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>TP=299 FP=0
+FN=1 TN=0
+SW=0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>at(tile,from)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>TP=5 FP=0
+FN=0 TN=0
+SW=0</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>TP=52 FP=0
+FN=6 TN=0
+SW=5</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>TP=48 FP=0
+FN=1 TN=0
+SW=1</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>TP=49 FP=0
+FN=2 TN=0
+SW=2</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>TP=162 FP=0
+FN=0 TN=0
+SW=0</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>TP=257 FP=0
+FN=1 TN=0
+SW=1</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>TP=207 FP=0
+FN=5 TN=0
+SW=3</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>TP=41 FP=0
+FN=0 TN=0
+SW=0</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>TP=289 FP=0
+FN=11 TN=0
+SW=6</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>TP=299 FP=0
+FN=1 TN=0
+SW=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>PRE</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>empty(to)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>TP=5 FP=0
 FN=0 TN=0</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>TP=57 FP=0
-FN=1 TN=0</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>TP=48 FP=0
-FN=1 TN=0</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>TP=48 FP=0
-FN=3 TN=0</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>TP=52 FP=0
+FN=6 TN=0</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>TP=47 FP=0
+FN=2 TN=0</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>TP=46 FP=0
+FN=5 TN=0</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>TP=162 FP=0
 FN=0 TN=0</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>TP=258 FP=0
-FN=0 TN=0</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>TP=211 FP=0
-FN=1 TN=0</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>TP=256 FP=0
+FN=2 TN=0</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>TP=206 FP=0
+FN=6 TN=0</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>TP=40 FP=0
 FN=1 TN=0</t>
         </is>
       </c>
-      <c r="K6" s="6" t="inlineStr">
-        <is>
-          <t>TP=297 FP=0
-FN=3 TN=0</t>
-        </is>
-      </c>
-      <c r="L6" s="6" t="inlineStr">
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>TP=282 FP=0
+FN=18 TN=0</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>TP=296 FP=0
+FN=4 TN=0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>ADD EFFECTS (in next state)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>at(tile,to)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>TP=5 FP=0
+FN=0 TN=0
+SW=0</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>TP=57 FP=0
+FN=1 TN=0
+SW=0</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>TP=49 FP=0
+FN=0 TN=0
+SW=0</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>TP=48 FP=0
+FN=3 TN=0
+SW=2</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>TP=162 FP=0
+FN=0 TN=0
+SW=0</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>TP=255 FP=0
+FN=3 TN=0
+SW=2</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>TP=209 FP=0
+FN=3 TN=0
+SW=3</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>TP=41 FP=0
+FN=0 TN=0
+SW=0</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>TP=290 FP=0
+FN=10 TN=0
+SW=7</t>
+        </is>
+      </c>
+      <c r="L11" s="6" t="inlineStr">
         <is>
           <t>TP=299 FP=0
-FN=1 TN=0</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>PRE</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>at(tile,from)</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
+FN=1 TN=0
+SW=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>empty(from)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>TP=5 FP=0
 FN=0 TN=0</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>TP=52 FP=0
 FN=6 TN=0</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>TP=48 FP=0
-FN=1 TN=0</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>TP=49 FP=0
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>TP=47 FP=0
 FN=2 TN=0</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>TP=46 FP=0
+FN=5 TN=0</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>TP=162 FP=0
 FN=0 TN=0</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>TP=257 FP=0
-FN=1 TN=0</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>TP=207 FP=0
-FN=5 TN=0</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>TP=41 FP=0
-FN=0 TN=0</t>
-        </is>
-      </c>
-      <c r="K7" s="6" t="inlineStr">
-        <is>
-          <t>TP=289 FP=0
-FN=11 TN=0</t>
-        </is>
-      </c>
-      <c r="L7" s="6" t="inlineStr">
-        <is>
-          <t>TP=299 FP=0
-FN=1 TN=0</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>PRE</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>empty(to)</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>TP=5 FP=0
-FN=0 TN=0</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>TP=52 FP=0
-FN=6 TN=0</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>TP=47 FP=0
-FN=2 TN=0</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>TP=46 FP=0
-FN=5 TN=0</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>TP=162 FP=0
-FN=0 TN=0</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>TP=256 FP=0
 FN=2 TN=0</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>TP=206 FP=0
 FN=6 TN=0</t>
         </is>
       </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>TP=40 FP=0
 FN=1 TN=0</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr">
+      <c r="K12" s="6" t="inlineStr">
         <is>
           <t>TP=282 FP=0
 FN=18 TN=0</t>
         </is>
       </c>
-      <c r="L8" s="6" t="inlineStr">
+      <c r="L12" s="6" t="inlineStr">
         <is>
           <t>TP=296 FP=0
 FN=4 TN=0</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>ADD EFFECTS (in next state)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>at(tile,to)</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>TP=5 FP=0
-FN=0 TN=0</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>TP=57 FP=0
-FN=1 TN=0</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>TP=49 FP=0
-FN=0 TN=0</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>TP=48 FP=0
-FN=3 TN=0</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>TP=162 FP=0
-FN=0 TN=0</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>TP=255 FP=0
-FN=3 TN=0</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>TP=209 FP=0
-FN=3 TN=0</t>
-        </is>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>TP=41 FP=0
-FN=0 TN=0</t>
-        </is>
-      </c>
-      <c r="K11" s="6" t="inlineStr">
-        <is>
-          <t>TP=290 FP=0
-FN=10 TN=0</t>
-        </is>
-      </c>
-      <c r="L11" s="6" t="inlineStr">
-        <is>
-          <t>TP=299 FP=0
-FN=1 TN=0</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>empty(from)</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>TP=5 FP=0
-FN=0 TN=0</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>TP=52 FP=0
-FN=6 TN=0</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>TP=47 FP=0
-FN=2 TN=0</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>TP=46 FP=0
-FN=5 TN=0</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>TP=162 FP=0
-FN=0 TN=0</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>TP=256 FP=0
-FN=2 TN=0</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="inlineStr">
-        <is>
-          <t>TP=206 FP=0
-FN=6 TN=0</t>
-        </is>
-      </c>
-      <c r="J12" s="6" t="inlineStr">
-        <is>
-          <t>TP=40 FP=0
-FN=1 TN=0</t>
-        </is>
-      </c>
-      <c r="K12" s="6" t="inlineStr">
-        <is>
-          <t>TP=282 FP=0
-FN=18 TN=0</t>
-        </is>
-      </c>
-      <c r="L12" s="6" t="inlineStr">
-        <is>
-          <t>TP=296 FP=0
-FN=4 TN=0</t>
-        </is>
-      </c>
-    </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -1003,61 +1033,71 @@
       <c r="C15" s="5" t="inlineStr">
         <is>
           <t>TP=0 FP=0
-FN=0 TN=5</t>
+FN=0 TN=5
+SW=0</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
           <t>TP=0 FP=0
-FN=0 TN=58</t>
+FN=0 TN=58
+SW=0</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
           <t>TP=0 FP=0
-FN=0 TN=49</t>
+FN=0 TN=49
+SW=0</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
           <t>TP=0 FP=0
-FN=0 TN=51</t>
+FN=0 TN=51
+SW=0</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
           <t>TP=0 FP=0
-FN=0 TN=162</t>
+FN=0 TN=162
+SW=0</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
           <t>TP=0 FP=1
-FN=0 TN=257</t>
+FN=0 TN=257
+SW=1</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
           <t>TP=0 FP=0
-FN=0 TN=212</t>
+FN=0 TN=212
+SW=0</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
           <t>TP=0 FP=0
-FN=0 TN=41</t>
+FN=0 TN=41
+SW=0</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
           <t>TP=0 FP=2
-FN=0 TN=298</t>
+FN=0 TN=298
+SW=2</t>
         </is>
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
           <t>TP=0 FP=0
-FN=0 TN=300</t>
+FN=0 TN=300
+SW=0</t>
         </is>
       </c>
     </row>
@@ -1259,6 +1299,11 @@
           <t>FA %</t>
         </is>
       </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Non-FA %</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1286,6 +1331,11 @@
           <t>0.0%</t>
         </is>
       </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
@@ -1313,6 +1363,11 @@
           <t>83.6%</t>
         </is>
       </c>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>16.4%</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1340,6 +1395,11 @@
           <t>69.2%</t>
         </is>
       </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>30.8%</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
@@ -1367,6 +1427,11 @@
           <t>64.0%</t>
         </is>
       </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>36.0%</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1394,6 +1459,11 @@
           <t>100.0%</t>
         </is>
       </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
@@ -1421,6 +1491,11 @@
           <t>90.9%</t>
         </is>
       </c>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
@@ -1448,6 +1523,11 @@
           <t>91.9%</t>
         </is>
       </c>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>8.1%</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1475,6 +1555,11 @@
           <t>66.7%</t>
         </is>
       </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>33.3%</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
@@ -1502,6 +1587,11 @@
           <t>90.6%</t>
         </is>
       </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
+          <t>9.4%</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
@@ -1527,6 +1617,11 @@
       <c r="G15" s="11" t="inlineStr">
         <is>
           <t>92.1%</t>
+        </is>
+      </c>
+      <c r="H15" s="11" t="inlineStr">
+        <is>
+          <t>7.9%</t>
         </is>
       </c>
     </row>
@@ -1558,6 +1653,10 @@
       </c>
       <c r="G16" s="12">
         <f>IF(D16&gt;0,TEXT(E16/D16*100,"0.0")&amp;"%","0%")</f>
+        <v/>
+      </c>
+      <c r="H16" s="12">
+        <f>IF(D16&gt;0,TEXT(F16/D16*100,"0.0")&amp;"%","0%")</f>
         <v/>
       </c>
     </row>

</xml_diff>